<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-05-20]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="instrumentos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cashflows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="instrumentos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cashflows" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,52 +418,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>maturity_date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ref_base_date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>cer_base_value</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>vn_base</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>base_precio</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>coupon_rate_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>coupon_freq</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>settle_rule</t>
         </is>
@@ -499,11 +487,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>652.7727190000001</v>
+        <v>651.898062</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -625,11 +613,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>661.1806779999999</v>
+        <v>659.678896</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -835,11 +823,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>652.7727190000001</v>
+        <v>651.898062</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -877,11 +865,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>652.7727190000001</v>
+        <v>651.898062</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -1087,11 +1075,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>732.635161</v>
+        <v>721.585027</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
@@ -1129,11 +1117,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>732.635161</v>
+        <v>721.585027</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1213,11 +1201,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2021-12-03</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>37.631094</v>
+        <v>37.587966</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
@@ -1255,11 +1243,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2022-05-13</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>46.913002</v>
+        <v>46.710616</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1297,11 +1285,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>732.635161</v>
+        <v>721.585027</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
@@ -1420,17 +1408,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>fecha</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>monto</t>
         </is>

</xml_diff>

<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-05-29]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X29Y6</t>
+          <t>X31L6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,16 +482,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>651.898062</v>
+        <v>685.550612</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X31L6</t>
+          <t>X30S6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -524,16 +524,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>685.550612</v>
+        <v>715.715236</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -556,7 +556,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,16 +566,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>715.715236</v>
+        <v>659.678896</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -598,26 +598,26 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZX26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LECER</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>659.678896</v>
+        <v>200.388015</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZX26</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,16 +650,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2024-10-17</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>200.388015</v>
+        <v>480.152578</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -692,16 +692,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>480.152578</v>
+        <v>271.047556</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,16 +734,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>271.047556</v>
+        <v>361.317603</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -776,16 +776,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2024-05-06</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>361.317603</v>
+        <v>651.898062</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -808,7 +808,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -860,16 +860,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>651.898062</v>
+        <v>200.388015</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -892,7 +892,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -902,16 +902,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>200.388015</v>
+        <v>715.715236</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -944,16 +944,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>715.715236</v>
+        <v>271.047556</v>
       </c>
       <c r="F13" t="n">
         <v>100</v>
@@ -976,7 +976,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -986,16 +986,16 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>271.047556</v>
+        <v>200.388015</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1018,7 +1018,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,16 +1028,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>200.388015</v>
+        <v>721.585027</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1060,7 +1060,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1102,26 +1102,26 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BONCER_ZC</t>
+          <t>BONCER_COUPON</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>721.585027</v>
+        <v>113.059645</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1130,10 +1130,10 @@
         <v>100</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1154,16 +1154,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>113.059645</v>
+        <v>37.587966</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1172,7 +1172,7 @@
         <v>100</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I18" t="n">
         <v>2</v>
@@ -1186,7 +1186,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1196,16 +1196,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2021-12-02</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>37.587966</v>
+        <v>46.710616</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
@@ -1214,7 +1214,7 @@
         <v>100</v>
       </c>
       <c r="H19" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I19" t="n">
         <v>2</v>
@@ -1228,26 +1228,26 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BONCER_COUPON</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>46.710616</v>
+        <v>721.585027</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1256,10 +1256,10 @@
         <v>100</v>
       </c>
       <c r="H20" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1270,7 +1270,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1280,16 +1280,16 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>721.585027</v>
+        <v>765.518009</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
@@ -1312,7 +1312,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1322,16 +1322,16 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>765.518009</v>
+        <v>756.63849</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>
@@ -1346,48 +1346,6 @@
         <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
-        <is>
-          <t>business_days_before:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>BONCER_ZC</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>756.63849</v>
-      </c>
-      <c r="F23" t="n">
-        <v>100</v>
-      </c>
-      <c r="G23" t="n">
-        <v>100</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="inlineStr">
         <is>
           <t>business_days_before:10</t>
         </is>
@@ -1404,7 +1362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1427,12 +1385,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X29Y6</t>
+          <t>X31L6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1442,12 +1400,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X31L6</t>
+          <t>X30S6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1457,12 +1415,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1472,12 +1430,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZX26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1487,12 +1445,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZX26</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1502,12 +1460,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1517,12 +1475,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1532,12 +1490,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1547,12 +1505,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1562,12 +1520,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1577,12 +1535,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1592,12 +1550,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1607,12 +1565,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1622,12 +1580,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1637,12 +1595,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1652,16 +1610,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1672,7 +1630,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1687,7 +1645,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1702,7 +1660,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1717,7 +1675,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1732,7 +1690,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1747,26 +1705,26 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>101</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="25">
@@ -1777,7 +1735,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1792,7 +1750,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2022-11-09</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1807,7 +1765,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1822,7 +1780,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1837,7 +1795,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1852,7 +1810,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1867,7 +1825,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1882,7 +1840,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1897,7 +1855,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1912,7 +1870,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-05-09</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1927,7 +1885,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2027-05-09</t>
+          <t>2027-11-09</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1942,7 +1900,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2027-11-09</t>
+          <t>2028-05-09</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1957,26 +1915,26 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2028-05-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1.125</v>
+        <v>101.125</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2022-05-30</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>101.125</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="39">
@@ -1987,7 +1945,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2022-05-30</t>
+          <t>2022-11-30</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -2002,7 +1960,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2023-05-30</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -2017,7 +1975,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2023-05-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -2032,7 +1990,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2023-11-30</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2047,7 +2005,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2062,7 +2020,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2077,7 +2035,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2092,7 +2050,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2107,7 +2065,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2122,7 +2080,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-30</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -2137,7 +2095,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2027-05-30</t>
+          <t>2027-11-30</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2152,7 +2110,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2027-11-30</t>
+          <t>2028-05-30</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2167,7 +2125,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2028-05-30</t>
+          <t>2028-11-30</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2182,7 +2140,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2028-11-30</t>
+          <t>2029-05-30</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2197,7 +2155,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2029-05-30</t>
+          <t>2029-11-30</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2212,7 +2170,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2029-11-30</t>
+          <t>2030-05-30</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2227,7 +2185,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2030-05-30</t>
+          <t>2030-11-30</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -2242,7 +2200,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2030-11-30</t>
+          <t>2031-05-30</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2257,37 +2215,37 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2031-05-30</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1.25</v>
+        <v>101.25</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>101.25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -2297,30 +2255,15 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-06-25]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>767.0346919999999</v>
+        <v>761.505166</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>756.63849</v>
+        <v>746.3809230000001</v>
       </c>
       <c r="F22" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-06-30]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,7 +598,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZX26</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -608,16 +608,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2024-10-17</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>200.388015</v>
+        <v>480.152578</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,16 +650,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>480.152578</v>
+        <v>271.047556</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -692,16 +692,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>271.047556</v>
+        <v>361.317603</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,16 +734,16 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2024-05-06</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>361.317603</v>
+        <v>651.898062</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -808,7 +808,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -818,16 +818,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>651.898062</v>
+        <v>200.388015</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -860,16 +860,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>200.388015</v>
+        <v>715.715236</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -892,7 +892,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -902,16 +902,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>715.715236</v>
+        <v>271.047556</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -944,16 +944,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>271.047556</v>
+        <v>200.388015</v>
       </c>
       <c r="F13" t="n">
         <v>100</v>
@@ -976,7 +976,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -986,16 +986,16 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>200.388015</v>
+        <v>721.585027</v>
       </c>
       <c r="F14" t="n">
         <v>100</v>
@@ -1018,7 +1018,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1060,26 +1060,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BONCER_ZC</t>
+          <t>BONCER_COUPON</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>721.585027</v>
+        <v>113.059645</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
@@ -1088,10 +1088,10 @@
         <v>100</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1112,16 +1112,16 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>113.059645</v>
+        <v>37.587966</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1130,7 +1130,7 @@
         <v>100</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I17" t="n">
         <v>2</v>
@@ -1144,7 +1144,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1154,16 +1154,16 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2021-12-02</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>37.587966</v>
+        <v>46.710616</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1172,7 +1172,7 @@
         <v>100</v>
       </c>
       <c r="H18" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I18" t="n">
         <v>2</v>
@@ -1186,26 +1186,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BONCER_COUPON</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>46.710616</v>
+        <v>721.585027</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
@@ -1214,10 +1214,10 @@
         <v>100</v>
       </c>
       <c r="H19" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1238,16 +1238,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>721.585027</v>
+        <v>761.505166</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1270,7 +1270,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1280,16 +1280,16 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>761.505166</v>
+        <v>746.3809230000001</v>
       </c>
       <c r="F21" t="n">
         <v>100</v>
@@ -1304,48 +1304,6 @@
         <v>0</v>
       </c>
       <c r="J21" t="inlineStr">
-        <is>
-          <t>business_days_before:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>BONCER_ZC</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>746.3809230000001</v>
-      </c>
-      <c r="F22" t="n">
-        <v>100</v>
-      </c>
-      <c r="G22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="inlineStr">
         <is>
           <t>business_days_before:10</t>
         </is>
@@ -1362,7 +1320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1430,12 +1388,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZX26</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1445,12 +1403,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1460,12 +1418,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1475,12 +1433,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1490,12 +1448,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1505,12 +1463,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1520,12 +1478,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1535,12 +1493,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1550,12 +1508,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1565,12 +1523,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1580,12 +1538,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1595,16 +1553,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1615,7 +1573,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1630,7 +1588,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1645,7 +1603,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1660,7 +1618,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1675,7 +1633,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1690,26 +1648,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>101</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="24">
@@ -1720,7 +1678,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1735,7 +1693,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2022-11-09</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1750,7 +1708,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1765,7 +1723,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1780,7 +1738,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1795,7 +1753,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1810,7 +1768,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1825,7 +1783,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1840,7 +1798,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1855,7 +1813,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-05-09</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1870,7 +1828,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2027-05-09</t>
+          <t>2027-11-09</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1885,7 +1843,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2027-11-09</t>
+          <t>2028-05-09</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1900,26 +1858,26 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2028-05-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.125</v>
+        <v>101.125</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2022-05-30</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>101.125</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="38">
@@ -1930,7 +1888,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2022-05-30</t>
+          <t>2022-11-30</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1945,7 +1903,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2023-05-30</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1960,7 +1918,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2023-05-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1975,7 +1933,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2023-11-30</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1990,7 +1948,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -2005,7 +1963,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2020,7 +1978,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -2035,7 +1993,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2050,7 +2008,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2065,7 +2023,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-30</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2080,7 +2038,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2027-05-30</t>
+          <t>2027-11-30</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -2095,7 +2053,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2027-11-30</t>
+          <t>2028-05-30</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2110,7 +2068,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2028-05-30</t>
+          <t>2028-11-30</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2125,7 +2083,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2028-11-30</t>
+          <t>2029-05-30</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2140,7 +2098,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2029-05-30</t>
+          <t>2029-11-30</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2155,7 +2113,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2029-11-30</t>
+          <t>2030-05-30</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2170,7 +2128,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2030-05-30</t>
+          <t>2030-11-30</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2185,7 +2143,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2030-11-30</t>
+          <t>2031-05-30</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -2200,37 +2158,37 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2031-05-30</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1.25</v>
+        <v>101.25</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>101.25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -2240,30 +2198,15 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: actualizar BD BONOS CER.xlsx [2026-07-31]
</commit_message>
<xml_diff>
--- a/backend/data/BD BONOS CER.xlsx
+++ b/backend/data/BD BONOS CER.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X31L6</t>
+          <t>X30S6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -482,16 +482,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>685.550612</v>
+        <v>715.715236</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
@@ -514,7 +514,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -524,16 +524,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>715.715236</v>
+        <v>659.678896</v>
       </c>
       <c r="F3" t="n">
         <v>100</v>
@@ -556,26 +556,26 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LECER</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
+          <t>2024-10-17</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>659.678896</v>
+        <v>480.152578</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
@@ -598,7 +598,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -608,16 +608,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>480.152578</v>
+        <v>271.047556</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,16 +650,16 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-05-06</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>271.047556</v>
+        <v>361.317603</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -682,7 +682,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -692,16 +692,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2024-05-06</t>
+          <t>2025-11-12</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>361.317603</v>
+        <v>651.898062</v>
       </c>
       <c r="F7" t="n">
         <v>100</v>
@@ -724,7 +724,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -766,7 +766,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -776,16 +776,16 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2025-11-12</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>651.898062</v>
+        <v>200.388015</v>
       </c>
       <c r="F9" t="n">
         <v>100</v>
@@ -808,7 +808,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -818,16 +818,16 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>200.388015</v>
+        <v>715.715236</v>
       </c>
       <c r="F10" t="n">
         <v>100</v>
@@ -850,7 +850,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -860,16 +860,16 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>715.715236</v>
+        <v>271.047556</v>
       </c>
       <c r="F11" t="n">
         <v>100</v>
@@ -892,7 +892,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -902,16 +902,16 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2024-03-01</t>
+          <t>2024-01-18</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>271.047556</v>
+        <v>200.388015</v>
       </c>
       <c r="F12" t="n">
         <v>100</v>
@@ -934,7 +934,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -944,16 +944,16 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2024-01-18</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>200.388015</v>
+        <v>721.585027</v>
       </c>
       <c r="F13" t="n">
         <v>100</v>
@@ -976,7 +976,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1018,26 +1018,26 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BONCER_ZC</t>
+          <t>BONCER_COUPON</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2023-07-18</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>721.585027</v>
+        <v>113.059645</v>
       </c>
       <c r="F15" t="n">
         <v>100</v>
@@ -1046,10 +1046,10 @@
         <v>100</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1070,16 +1070,16 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2023-07-18</t>
+          <t>2021-12-02</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>113.059645</v>
+        <v>37.587966</v>
       </c>
       <c r="F16" t="n">
         <v>100</v>
@@ -1088,7 +1088,7 @@
         <v>100</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I16" t="n">
         <v>2</v>
@@ -1102,7 +1102,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1112,16 +1112,16 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2021-12-02</t>
+          <t>2022-05-11</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>37.587966</v>
+        <v>46.710616</v>
       </c>
       <c r="F17" t="n">
         <v>100</v>
@@ -1130,7 +1130,7 @@
         <v>100</v>
       </c>
       <c r="H17" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="I17" t="n">
         <v>2</v>
@@ -1144,26 +1144,26 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BONCER_COUPON</t>
+          <t>BONCER_ZC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2022-05-11</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>46.710616</v>
+        <v>721.585027</v>
       </c>
       <c r="F18" t="n">
         <v>100</v>
@@ -1172,10 +1172,10 @@
         <v>100</v>
       </c>
       <c r="H18" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1196,16 +1196,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>721.585027</v>
+        <v>761.505166</v>
       </c>
       <c r="F19" t="n">
         <v>100</v>
@@ -1228,7 +1228,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1238,16 +1238,16 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>761.505166</v>
+        <v>746.3809230000001</v>
       </c>
       <c r="F20" t="n">
         <v>100</v>
@@ -1262,48 +1262,6 @@
         <v>0</v>
       </c>
       <c r="J20" t="inlineStr">
-        <is>
-          <t>business_days_before:10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>BONCER_ZC</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>746.3809230000001</v>
-      </c>
-      <c r="F21" t="n">
-        <v>100</v>
-      </c>
-      <c r="G21" t="n">
-        <v>100</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="inlineStr">
         <is>
           <t>business_days_before:10</t>
         </is>
@@ -1320,7 +1278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1343,12 +1301,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>X31L6</t>
+          <t>X30S6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -1358,12 +1316,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>X30S6</t>
+          <t>X30N6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -1373,12 +1331,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>X30N6</t>
+          <t>TZXO6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1388,12 +1346,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TZXO6</t>
+          <t>TZXD6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1403,12 +1361,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TZXD6</t>
+          <t>TZXM7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2027-03-31</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1418,12 +1376,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TZXM7</t>
+          <t>TZXA7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-03-31</t>
+          <t>2027-04-30</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1433,12 +1391,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TZXA7</t>
+          <t>TZXY7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2027-04-30</t>
+          <t>2027-05-31</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1448,12 +1406,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TZXY7</t>
+          <t>TZX27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2027-05-31</t>
+          <t>2027-06-30</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1463,12 +1421,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TZX27</t>
+          <t>TZXS7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2027-09-30</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1478,12 +1436,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TZXS7</t>
+          <t>TZXD7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2027-09-30</t>
+          <t>2027-12-15</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1493,12 +1451,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TZXD7</t>
+          <t>TZX28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2027-12-15</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1508,12 +1466,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TZX28</t>
+          <t>TZXS8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2028-09-29</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1523,12 +1481,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TZXS8</t>
+          <t>TZXM9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2028-09-29</t>
+          <t>2029-03-28</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1538,16 +1496,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TZXM9</t>
+          <t>TX26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2029-03-28</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1558,7 +1516,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1573,7 +1531,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1588,7 +1546,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1603,7 +1561,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1618,7 +1576,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1633,26 +1591,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TX26</t>
+          <t>TX28</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2022-05-09</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>101</v>
+        <v>1.125</v>
       </c>
     </row>
     <row r="23">
@@ -1663,7 +1621,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2022-05-09</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1678,7 +1636,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2022-11-09</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1693,7 +1651,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-11-09</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1708,7 +1666,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2023-11-09</t>
+          <t>2024-05-09</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1723,7 +1681,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-05-09</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1738,7 +1696,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2025-05-09</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1753,7 +1711,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1768,7 +1726,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1783,7 +1741,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1798,7 +1756,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-05-09</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1813,7 +1771,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2027-05-09</t>
+          <t>2027-11-09</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1828,7 +1786,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2027-11-09</t>
+          <t>2028-05-09</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1843,26 +1801,26 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2028-05-09</t>
+          <t>2028-11-09</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.125</v>
+        <v>101.125</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TX28</t>
+          <t>TX31</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2028-11-09</t>
+          <t>2022-05-30</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>101.125</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="37">
@@ -1873,7 +1831,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2022-05-30</t>
+          <t>2022-11-30</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1888,7 +1846,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2023-05-30</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1903,7 +1861,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2023-05-30</t>
+          <t>2023-11-30</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1918,7 +1876,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2023-11-30</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1933,7 +1891,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1948,7 +1906,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1963,7 +1921,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1978,7 +1936,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1993,7 +1951,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2008,7 +1966,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2027-05-30</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -2023,7 +1981,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2027-05-30</t>
+          <t>2027-11-30</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2038,7 +1996,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2027-11-30</t>
+          <t>2028-05-30</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -2053,7 +2011,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2028-05-30</t>
+          <t>2028-11-30</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2068,7 +2026,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2028-11-30</t>
+          <t>2029-05-30</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -2083,7 +2041,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2029-05-30</t>
+          <t>2029-11-30</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -2098,7 +2056,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2029-11-30</t>
+          <t>2030-05-30</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -2113,7 +2071,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2030-05-30</t>
+          <t>2030-11-30</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -2128,7 +2086,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2030-11-30</t>
+          <t>2031-05-30</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -2143,37 +2101,37 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2031-05-30</t>
+          <t>2031-11-30</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.25</v>
+        <v>101.25</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TX31</t>
+          <t>TZXM8</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2031-11-30</t>
+          <t>2028-03-31</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>101.25</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TZXM8</t>
+          <t>TXM8</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2028-03-31</t>
+          <t>2028-06-30</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2183,30 +2141,15 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TXM8</t>
+          <t>TXM9</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2028-06-30</t>
+          <t>2029-06-29</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>TXM9</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>2029-06-29</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>